<commit_message>
Refactor ECG denoising model training and update annotations
- Updated JSON annotation file for ECG data with new flags and comments.
- Added new noise annotations and adjusted counts in the rpeakAnnotationCounts.
- Introduced a new Python script for training a ResUNet-based denoising autoencoder for ECG signals.
- Created a shell script to facilitate training with specified parameters.
- Removed unnecessary files and updated Excel records for noise indices.
- Enhanced logging and visualization capabilities in the training script.
</commit_message>
<xml_diff>
--- a/0_SELECT_ZIVE_DATA_2023/UPDATE_RECORDS_LIST_ADDING_ML_NOISES/visi_zive_irasai_annot - Darb.xlsx
+++ b/0_SELECT_ZIVE_DATA_2023/UPDATE_RECORDS_LIST_ADDING_ML_NOISES/visi_zive_irasai_annot - Darb.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kesju\DI\2025_ZIVEO\PROJECT_TRAIN_UNET\0_SELECT_ZIVE_DATA_2023\UPDATE_RECORDS_LIST_ADDING_ML_NOISES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEFEB5AB-2A92-42A4-975E-35CC1669E29B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F0776CF-AF66-4841-92CB-1DA43DDF2D1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="18600" windowHeight="9420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Zymejimas" sheetId="2" r:id="rId2"/>
+    <sheet name="Komentarai" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8685" uniqueCount="3870">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8688" uniqueCount="3872">
   <si>
     <t>filename</t>
   </si>
@@ -11645,6 +11646,12 @@
   </si>
   <si>
     <t>1630737.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1630768.486 </t>
+  </si>
+  <si>
+    <t>Norėčiau atkreipti dėmesį į 1630768.486 įrašą. Kelis kartus po skilvelinės ekstrasistolės šiame įraše stebime vadinamus "fusion beat" (susiliejęs kompleksas). Jį lemia tai, jog skilvelių depoliarizaciją lemia tiek neseniai buvusi skilvelinė ekstrasistolė, tiek iš sinusinio mazgo atėjęs impulsas ir šios dvi skilvelio aktyvacijos susilieja, todėl keičia morfologiją, palyginus su įprastu sinusiniu kompleksu, tačiau nėra platus kaip skilvelinė ekstrasistolė. Šiuo atveju tai nėra nei skilvelinė, nei prieširdinė ekstrasistolės, nei normalus QRS kompleksas. Tam, kad neklaidinti algoritmo pažymėjau juos U raide.</t>
   </si>
 </sst>
 </file>
@@ -11655,7 +11662,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -11673,6 +11680,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -11756,7 +11769,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -11787,11 +11800,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -11808,6 +11827,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -12101,7 +12124,7 @@
     <col min="3" max="3" width="13.6328125" style="17" customWidth="1"/>
     <col min="4" max="5" width="7.36328125" customWidth="1"/>
     <col min="6" max="6" width="9.26953125" customWidth="1"/>
-    <col min="7" max="7" width="12.6328125" customWidth="1"/>
+    <col min="7" max="7" width="16.54296875" customWidth="1"/>
     <col min="8" max="8" width="6.6328125" hidden="1" customWidth="1"/>
     <col min="9" max="10" width="6.7265625" style="10" customWidth="1"/>
     <col min="11" max="11" width="4.7265625" customWidth="1"/>
@@ -12117,9 +12140,9 @@
     <col min="21" max="21" width="6.26953125" style="11" customWidth="1"/>
     <col min="22" max="22" width="4.90625" style="11" customWidth="1"/>
     <col min="23" max="23" width="5.90625" style="11" customWidth="1"/>
-    <col min="24" max="24" width="9.81640625" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="13.1796875" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="12.08984375" style="12" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="9.81640625" customWidth="1"/>
+    <col min="25" max="25" width="13.1796875" customWidth="1"/>
+    <col min="26" max="26" width="12.08984375" style="12" customWidth="1"/>
     <col min="27" max="27" width="54.6328125" customWidth="1"/>
     <col min="28" max="28" width="28.81640625" customWidth="1"/>
     <col min="29" max="29" width="27.1796875" customWidth="1"/>
@@ -109150,4 +109173,31 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC8927EF-A8B6-4332-97A4-1580ECD6BC5E}">
+  <dimension ref="A2:B3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.36328125" customWidth="1"/>
+    <col min="2" max="2" width="128.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="80" x14ac:dyDescent="0.35">
+      <c r="A3" s="19" t="s">
+        <v>3870</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>3871</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>